<commit_message>
feat: scraper veille + 2 offres IPSA/IONIS + cron quotidien
- veille_scraper.py : scraping écoles + Google Jobs
- scraper_jobs.py : Playwright pour LinkedIn/WTTJ
- 2 offres cybersécurité IPSA (Ivry-sur-Seine)
- Excel avec suivi des statuts + tableau de bord
- Cron veille quotidienne 8h00 configuré
- Template email de prospection validé POC
</commit_message>
<xml_diff>
--- a/data/cyber-tech_prospection.xlsx
+++ b/data/cyber-tech_prospection.xlsx
@@ -20,7 +20,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="5">
+  <fonts count="6">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -47,6 +47,12 @@
       <name val="Calibri"/>
       <b val="1"/>
       <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="000563C1"/>
+      <sz val="10"/>
+      <u val="single"/>
     </font>
   </fonts>
   <fills count="3">
@@ -81,7 +87,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -92,6 +98,12 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -492,7 +504,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L1"/>
+  <dimension ref="A1:L5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="45" customWidth="1" min="1" max="1"/>
@@ -568,6 +580,122 @@
       <c r="L1" s="1" t="inlineStr">
         <is>
           <t>Notes</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="6" t="inlineStr">
+        <is>
+          <t>Enseignant-chercheur en Réseaux et Cybersécurité (Section CNU 27/61)</t>
+        </is>
+      </c>
+      <c r="B3" s="6" t="inlineStr">
+        <is>
+          <t>IPSA — IONIS Group</t>
+        </is>
+      </c>
+      <c r="C3" s="6" t="inlineStr">
+        <is>
+          <t>CDI — Temps plein</t>
+        </is>
+      </c>
+      <c r="D3" s="6" t="inlineStr">
+        <is>
+          <t>Réseaux, cybersécurité, enseignement supérieur</t>
+        </is>
+      </c>
+      <c r="E3" s="6" t="inlineStr">
+        <is>
+          <t>Bac+5 (Enseignant-chercheur)</t>
+        </is>
+      </c>
+      <c r="F3" s="6" t="inlineStr">
+        <is>
+          <t>Ivry-sur-Seine (94) — Île-de-France</t>
+        </is>
+      </c>
+      <c r="G3" s="6" t="inlineStr">
+        <is>
+          <t>2026-03-11</t>
+        </is>
+      </c>
+      <c r="H3" s="6" t="inlineStr">
+        <is>
+          <t>Non précisée</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>https://careers.werecruit.io/fr/ionis-group/offres/enseignant-chercheur-en-reseaux-et-cybersecurite-section-cnu-2761-2634c9</t>
+        </is>
+      </c>
+      <c r="J3" s="6" t="inlineStr"/>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>Non contacté</t>
+        </is>
+      </c>
+      <c r="L3" s="6" t="inlineStr">
+        <is>
+          <t>Poste d'enseignant-chercheur à l'IPSA (école d'ingénieurs du groupe IONIS). CDI temps plein.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>Enseignant en informatique, réseau et cybersécurité</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>IPSA — IONIS Group</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>CDI — Temps plein</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Informatique, réseaux, cybersécurité</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Bac+5 (Enseignant)</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>Ivry-sur-Seine (94) — Île-de-France</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>2026-02-23</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>Non précisée (début 01/09/2026)</t>
+        </is>
+      </c>
+      <c r="I5" s="7" t="inlineStr">
+        <is>
+          <t>https://careers.werecruit.io/fr/ionis-group/offres/enseignant-en-informatique-reseau-et-cybersecurite-0b2fc1</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr"/>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>Non contacté</t>
+        </is>
+      </c>
+      <c r="L5" s="6" t="inlineStr">
+        <is>
+          <t>Poste d'enseignant à l'IPSA. Début au 1er septembre 2026.</t>
         </is>
       </c>
     </row>
@@ -625,7 +753,7 @@
         </is>
       </c>
       <c r="B2" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -806,7 +934,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>15/06/2026 15:47</t>
+          <t>15/06/2026 16:11</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: POC email envoye + statut mis a jour
- Email de prospection envoye a rabih.zgheib@cyber-tech.me (POC)
- Statut offres passe a 'Email envoye dans offres.json
- Excel mis a jour
- Template email valide en POC
</commit_message>
<xml_diff>
--- a/data/cyber-tech_prospection.xlsx
+++ b/data/cyber-tech_prospection.xlsx
@@ -629,15 +629,19 @@
           <t>https://careers.werecruit.io/fr/ionis-group/offres/enseignant-chercheur-en-reseaux-et-cybersecurite-section-cnu-2761-2634c9</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="inlineStr">
+        <is>
+          <t>rabih.zgheib@cyber-tech.me (POC)</t>
+        </is>
+      </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
-          <t>Non contacté</t>
+          <t>Email envoyé</t>
         </is>
       </c>
       <c r="L3" s="6" t="inlineStr">
         <is>
-          <t>Poste d'enseignant-chercheur à l'IPSA (école d'ingénieurs du groupe IONIS). CDI temps plein.</t>
+          <t>Poste d'enseignant-chercheur à l'IPSA (école d'ingénieurs du groupe IONIS). CDI temps plein. | POC envoye le 15/06/2026 (validation en attente)</t>
         </is>
       </c>
     </row>
@@ -687,15 +691,19 @@
           <t>https://careers.werecruit.io/fr/ionis-group/offres/enseignant-en-informatique-reseau-et-cybersecurite-0b2fc1</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>rabih.zgheib@cyber-tech.me (POC)</t>
+        </is>
+      </c>
       <c r="K5" s="6" t="inlineStr">
         <is>
-          <t>Non contacté</t>
+          <t>Email envoyé</t>
         </is>
       </c>
       <c r="L5" s="6" t="inlineStr">
         <is>
-          <t>Poste d'enseignant à l'IPSA. Début au 1er septembre 2026.</t>
+          <t>Poste d'enseignant à l'IPSA. Début au 1er septembre 2026. | POC envoye le 15/06/2026 (validation en attente)</t>
         </is>
       </c>
     </row>
@@ -901,7 +909,7 @@
         </is>
       </c>
       <c r="B19" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="20">
@@ -923,7 +931,7 @@
         </is>
       </c>
       <c r="B21" s="4" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="22">
@@ -934,7 +942,7 @@
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>15/06/2026 16:11</t>
+          <t>15/06/2026 20:26</t>
         </is>
       </c>
     </row>

</xml_diff>